<commit_message>
big shift today. a lot of audio processing done harmonic and radar sound graphs
</commit_message>
<xml_diff>
--- a/practical/microphones.xlsx
+++ b/practical/microphones.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louis\source\repos\propeller-acoustics\practical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4B7DCC-A33A-4705-8F2B-3012DEAA819C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45191A57-25C8-488E-8D1E-5C06B56EF8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{C9460D7B-CB41-44A6-BCFB-2C82C87EA7E5}"/>
+    <workbookView xWindow="825" yWindow="2730" windowWidth="21600" windowHeight="11333" activeTab="1" xr2:uid="{C9460D7B-CB41-44A6-BCFB-2C82C87EA7E5}"/>
   </bookViews>
   <sheets>
     <sheet name="position" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
   <si>
     <t>microphone</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>distance</t>
-  </si>
-  <si>
-    <t>14οο</t>
   </si>
   <si>
     <t>yes</t>
@@ -73,9 +70,6 @@
   </si>
   <si>
     <t>1p</t>
-  </si>
-  <si>
-    <t>ηοο</t>
   </si>
   <si>
     <t>2f</t>
@@ -265,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
@@ -296,7 +290,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
@@ -658,7 +651,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -675,7 +668,7 @@
         <v>1270</v>
       </c>
       <c r="E2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -692,7 +685,7 @@
         <v>1270</v>
       </c>
       <c r="E3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -709,7 +702,7 @@
         <v>1270</v>
       </c>
       <c r="E4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -726,7 +719,7 @@
         <v>1270</v>
       </c>
       <c r="E5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -743,7 +736,7 @@
         <v>1270</v>
       </c>
       <c r="E6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -760,7 +753,7 @@
         <v>1270</v>
       </c>
       <c r="E7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -777,7 +770,7 @@
         <v>1270</v>
       </c>
       <c r="E8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1048576" spans="5:5" x14ac:dyDescent="0.45">
@@ -797,95 +790,95 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>13</v>
-      </c>
       <c r="F2" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="L2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="M2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="N2" s="7" t="s">
         <v>22</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16.899999999999999" thickBot="1" x14ac:dyDescent="0.5">
@@ -925,10 +918,10 @@
       <c r="L4" s="9">
         <v>0</v>
       </c>
-      <c r="M4" s="13">
+      <c r="M4" s="12">
         <v>250</v>
       </c>
-      <c r="N4" s="13">
+      <c r="N4" s="12">
         <v>0</v>
       </c>
     </row>
@@ -969,10 +962,10 @@
       <c r="L5" s="9">
         <v>0</v>
       </c>
-      <c r="M5" s="14">
+      <c r="M5" s="13">
         <v>280</v>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="13">
         <v>-0.01</v>
       </c>
     </row>
@@ -1013,10 +1006,10 @@
       <c r="L6" s="9">
         <v>-0.01</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="13">
         <v>315</v>
       </c>
-      <c r="N6" s="13">
+      <c r="N6" s="12">
         <v>-0.02</v>
       </c>
     </row>
@@ -1057,10 +1050,10 @@
       <c r="L7" s="9">
         <v>0.01</v>
       </c>
-      <c r="M7" s="14">
+      <c r="M7" s="13">
         <v>355</v>
       </c>
-      <c r="N7" s="13">
+      <c r="N7" s="12">
         <v>-0.03</v>
       </c>
     </row>
@@ -1101,10 +1094,10 @@
       <c r="L8" s="9">
         <v>-0.01</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="13">
         <v>400</v>
       </c>
-      <c r="N8" s="13">
+      <c r="N8" s="12">
         <v>-0.04</v>
       </c>
     </row>
@@ -1145,10 +1138,10 @@
       <c r="L9" s="9">
         <v>-0.02</v>
       </c>
-      <c r="M9" s="14">
+      <c r="M9" s="13">
         <v>450</v>
       </c>
-      <c r="N9" s="13">
+      <c r="N9" s="12">
         <v>-0.05</v>
       </c>
     </row>
@@ -1189,10 +1182,10 @@
       <c r="L10" s="9">
         <v>-0.02</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="13">
         <v>500</v>
       </c>
-      <c r="N10" s="13">
+      <c r="N10" s="12">
         <v>-0.05</v>
       </c>
     </row>
@@ -1233,10 +1226,10 @@
       <c r="L11" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M11" s="13">
+      <c r="M11" s="12">
         <v>560</v>
       </c>
-      <c r="N11" s="13">
+      <c r="N11" s="12">
         <v>-0.06</v>
       </c>
     </row>
@@ -1277,10 +1270,10 @@
       <c r="L12" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="12">
         <v>630</v>
       </c>
-      <c r="N12" s="13">
+      <c r="N12" s="12">
         <v>-7.0000000000000007E-2</v>
       </c>
     </row>
@@ -1321,10 +1314,10 @@
       <c r="L13" s="9">
         <v>-0.02</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="12">
         <v>710</v>
       </c>
-      <c r="N13" s="13">
+      <c r="N13" s="12">
         <v>-7.0000000000000007E-2</v>
       </c>
     </row>
@@ -1365,10 +1358,10 @@
       <c r="L14" s="9">
         <v>-0.04</v>
       </c>
-      <c r="M14" s="13">
+      <c r="M14" s="12">
         <v>800</v>
       </c>
-      <c r="N14" s="13">
+      <c r="N14" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1409,10 +1402,10 @@
       <c r="L15" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M15" s="13">
+      <c r="M15" s="12">
         <v>900</v>
       </c>
-      <c r="N15" s="13">
+      <c r="N15" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1453,10 +1446,10 @@
       <c r="L16" s="9">
         <v>-0.04</v>
       </c>
-      <c r="M16" s="13">
+      <c r="M16" s="12">
         <v>1000</v>
       </c>
-      <c r="N16" s="13">
+      <c r="N16" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1497,10 +1490,10 @@
       <c r="L17" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M17" s="13">
+      <c r="M17" s="12">
         <v>1120</v>
       </c>
-      <c r="N17" s="13">
+      <c r="N17" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1541,10 +1534,10 @@
       <c r="L18" s="9">
         <v>-0.04</v>
       </c>
-      <c r="M18" s="13">
+      <c r="M18" s="12">
         <v>1250</v>
       </c>
-      <c r="N18" s="13">
+      <c r="N18" s="12">
         <v>-0.09</v>
       </c>
     </row>
@@ -1567,8 +1560,8 @@
       <c r="F19" s="4">
         <v>-0.02</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>4</v>
+      <c r="G19" s="3">
+        <v>1400</v>
       </c>
       <c r="H19" s="4">
         <v>-0.03</v>
@@ -1585,10 +1578,10 @@
       <c r="L19" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M19" s="13">
+      <c r="M19" s="12">
         <v>1400</v>
       </c>
-      <c r="N19" s="13">
+      <c r="N19" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1629,10 +1622,10 @@
       <c r="L20" s="10">
         <v>-0.03</v>
       </c>
-      <c r="M20" s="13">
+      <c r="M20" s="12">
         <v>1600</v>
       </c>
-      <c r="N20" s="13">
+      <c r="N20" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1673,10 +1666,10 @@
       <c r="L21" s="9">
         <v>-0.03</v>
       </c>
-      <c r="M21" s="13">
+      <c r="M21" s="12">
         <v>1800</v>
       </c>
-      <c r="N21" s="13">
+      <c r="N21" s="12">
         <v>-0.08</v>
       </c>
     </row>
@@ -1717,10 +1710,10 @@
       <c r="L22" s="9">
         <v>-0.02</v>
       </c>
-      <c r="M22" s="13">
+      <c r="M22" s="12">
         <v>2000</v>
       </c>
-      <c r="N22" s="13">
+      <c r="N22" s="12">
         <v>-7.0000000000000007E-2</v>
       </c>
     </row>
@@ -1761,10 +1754,10 @@
       <c r="L23" s="9">
         <v>-0.01</v>
       </c>
-      <c r="M23" s="13">
+      <c r="M23" s="12">
         <v>2240</v>
       </c>
-      <c r="N23" s="13">
+      <c r="N23" s="12">
         <v>-7.0000000000000007E-2</v>
       </c>
     </row>
@@ -1805,10 +1798,10 @@
       <c r="L24" s="9">
         <v>0</v>
       </c>
-      <c r="M24" s="13">
+      <c r="M24" s="12">
         <v>2500</v>
       </c>
-      <c r="N24" s="13">
+      <c r="N24" s="12">
         <v>-0.06</v>
       </c>
     </row>
@@ -1849,10 +1842,10 @@
       <c r="L25" s="9">
         <v>-0.01</v>
       </c>
-      <c r="M25" s="13">
+      <c r="M25" s="12">
         <v>2800</v>
       </c>
-      <c r="N25" s="13">
+      <c r="N25" s="12">
         <v>-0.04</v>
       </c>
     </row>
@@ -1893,10 +1886,10 @@
       <c r="L26" s="9">
         <v>0.01</v>
       </c>
-      <c r="M26" s="14">
+      <c r="M26" s="13">
         <v>3150</v>
       </c>
-      <c r="N26" s="13">
+      <c r="N26" s="12">
         <v>-0.03</v>
       </c>
     </row>
@@ -1937,10 +1930,10 @@
       <c r="L27" s="11">
         <v>0.03</v>
       </c>
-      <c r="M27" s="13">
+      <c r="M27" s="12">
         <v>3550</v>
       </c>
-      <c r="N27" s="13">
+      <c r="N27" s="12">
         <v>0</v>
       </c>
     </row>
@@ -1981,10 +1974,10 @@
       <c r="L28" s="9">
         <v>0.06</v>
       </c>
-      <c r="M28" s="14">
+      <c r="M28" s="13">
         <v>4000</v>
       </c>
-      <c r="N28" s="13">
+      <c r="N28" s="12">
         <v>0.03</v>
       </c>
     </row>
@@ -2025,10 +2018,10 @@
       <c r="L29" s="10">
         <v>0.1</v>
       </c>
-      <c r="M29" s="13">
+      <c r="M29" s="12">
         <v>4500</v>
       </c>
-      <c r="N29" s="13">
+      <c r="N29" s="12">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
@@ -2069,10 +2062,10 @@
       <c r="L30" s="9">
         <v>0.13</v>
       </c>
-      <c r="M30" s="13">
+      <c r="M30" s="12">
         <v>5000</v>
       </c>
-      <c r="N30" s="13">
+      <c r="N30" s="12">
         <v>0.11</v>
       </c>
     </row>
@@ -2113,10 +2106,10 @@
       <c r="L31" s="9">
         <v>0.18</v>
       </c>
-      <c r="M31" s="13">
+      <c r="M31" s="12">
         <v>5600</v>
       </c>
-      <c r="N31" s="13">
+      <c r="N31" s="12">
         <v>0.17</v>
       </c>
     </row>
@@ -2157,10 +2150,10 @@
       <c r="L32" s="9">
         <v>0.2</v>
       </c>
-      <c r="M32" s="13">
+      <c r="M32" s="12">
         <v>6300</v>
       </c>
-      <c r="N32" s="13">
+      <c r="N32" s="12">
         <v>0.24</v>
       </c>
     </row>
@@ -2171,8 +2164,8 @@
       <c r="B33" s="4">
         <v>0.28999999999999998</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>12</v>
+      <c r="C33" s="3">
+        <v>7100</v>
       </c>
       <c r="D33" s="4">
         <v>0.19</v>
@@ -2201,10 +2194,10 @@
       <c r="L33" s="9">
         <v>0.3</v>
       </c>
-      <c r="M33" s="13">
+      <c r="M33" s="12">
         <v>7100</v>
       </c>
-      <c r="N33" s="13">
+      <c r="N33" s="12">
         <v>0.35</v>
       </c>
     </row>
@@ -2245,10 +2238,10 @@
       <c r="L34" s="9">
         <v>0.31</v>
       </c>
-      <c r="M34" s="13">
+      <c r="M34" s="12">
         <v>8000</v>
       </c>
-      <c r="N34" s="13">
+      <c r="N34" s="12">
         <v>0.47</v>
       </c>
     </row>
@@ -2289,10 +2282,10 @@
       <c r="L35" s="9">
         <v>0.22</v>
       </c>
-      <c r="M35" s="13">
+      <c r="M35" s="12">
         <v>9000</v>
       </c>
-      <c r="N35" s="13">
+      <c r="N35" s="12">
         <v>0.6</v>
       </c>
     </row>
@@ -2333,10 +2326,10 @@
       <c r="L36" s="9">
         <v>0.4</v>
       </c>
-      <c r="M36" s="13">
+      <c r="M36" s="12">
         <v>10000</v>
       </c>
-      <c r="N36" s="13">
+      <c r="N36" s="12">
         <v>0.68</v>
       </c>
     </row>
@@ -2377,10 +2370,10 @@
       <c r="L37" s="9">
         <v>0.34</v>
       </c>
-      <c r="M37" s="13">
+      <c r="M37" s="12">
         <v>11200</v>
       </c>
-      <c r="N37" s="13">
+      <c r="N37" s="12">
         <v>0.8</v>
       </c>
     </row>
@@ -2421,10 +2414,10 @@
       <c r="L38" s="9">
         <v>0.28000000000000003</v>
       </c>
-      <c r="M38" s="14">
+      <c r="M38" s="13">
         <v>12500</v>
       </c>
-      <c r="N38" s="13">
+      <c r="N38" s="12">
         <v>0.93</v>
       </c>
     </row>
@@ -2465,10 +2458,10 @@
       <c r="L39" s="9">
         <v>0.22</v>
       </c>
-      <c r="M39" s="13">
+      <c r="M39" s="12">
         <v>14000</v>
       </c>
-      <c r="N39" s="13">
+      <c r="N39" s="12">
         <v>1.1399999999999999</v>
       </c>
     </row>
@@ -2509,10 +2502,10 @@
       <c r="L40" s="9">
         <v>0</v>
       </c>
-      <c r="M40" s="13">
+      <c r="M40" s="12">
         <v>16000</v>
       </c>
-      <c r="N40" s="13">
+      <c r="N40" s="12">
         <v>1.35</v>
       </c>
     </row>
@@ -2553,10 +2546,10 @@
       <c r="L41" s="9">
         <v>-0.38</v>
       </c>
-      <c r="M41" s="13">
+      <c r="M41" s="12">
         <v>18000</v>
       </c>
-      <c r="N41" s="13">
+      <c r="N41" s="12">
         <v>1.51</v>
       </c>
     </row>
@@ -2597,10 +2590,10 @@
       <c r="L42" s="10">
         <v>-1.01</v>
       </c>
-      <c r="M42" s="13">
+      <c r="M42" s="12">
         <v>20000</v>
       </c>
-      <c r="N42" s="13">
+      <c r="N42" s="12">
         <v>1.26</v>
       </c>
     </row>
@@ -2641,10 +2634,10 @@
       <c r="L43" s="9">
         <v>-2.0299999999999998</v>
       </c>
-      <c r="M43" s="13">
+      <c r="M43" s="12">
         <v>22400</v>
       </c>
-      <c r="N43" s="13">
+      <c r="N43" s="12">
         <v>0.28000000000000003</v>
       </c>
     </row>
@@ -2685,10 +2678,10 @@
       <c r="L44" s="9">
         <v>-3.46</v>
       </c>
-      <c r="M44" s="13">
+      <c r="M44" s="12">
         <v>25000</v>
       </c>
-      <c r="N44" s="13">
+      <c r="N44" s="12">
         <v>-1.98</v>
       </c>
     </row>
@@ -2729,10 +2722,10 @@
       <c r="L45" s="9">
         <v>-5.19</v>
       </c>
-      <c r="M45" s="13">
+      <c r="M45" s="12">
         <v>28000</v>
       </c>
-      <c r="N45" s="13">
+      <c r="N45" s="12">
         <v>-5.31</v>
       </c>
     </row>
@@ -2773,10 +2766,10 @@
       <c r="L46" s="9">
         <v>-5.94</v>
       </c>
-      <c r="M46" s="13">
+      <c r="M46" s="12">
         <v>31500</v>
       </c>
-      <c r="N46" s="13">
+      <c r="N46" s="12">
         <v>-8.06</v>
       </c>
     </row>
@@ -2817,10 +2810,10 @@
       <c r="L47" s="10">
         <v>-4.78</v>
       </c>
-      <c r="M47" s="13">
+      <c r="M47" s="12">
         <v>35500</v>
       </c>
-      <c r="N47" s="13">
+      <c r="N47" s="12">
         <v>-7.13</v>
       </c>
     </row>
@@ -2861,10 +2854,10 @@
       <c r="L48" s="10">
         <v>-6.88</v>
       </c>
-      <c r="M48" s="13">
+      <c r="M48" s="12">
         <v>40000</v>
       </c>
-      <c r="N48" s="13">
+      <c r="N48" s="12">
         <v>-9.5500000000000007</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finally fixed the microphones
</commit_message>
<xml_diff>
--- a/practical/microphones.xlsx
+++ b/practical/microphones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louis\source\repos\propeller-acoustics\practical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45191A57-25C8-488E-8D1E-5C06B56EF8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B859B7-4CD3-44F3-B93A-2B0CE4C95B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="825" yWindow="2730" windowWidth="21600" windowHeight="11333" activeTab="1" xr2:uid="{C9460D7B-CB41-44A6-BCFB-2C82C87EA7E5}"/>
+    <workbookView xWindow="4455" yWindow="2258" windowWidth="21600" windowHeight="11332" xr2:uid="{C9460D7B-CB41-44A6-BCFB-2C82C87EA7E5}"/>
   </bookViews>
   <sheets>
     <sheet name="position" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>microphone</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>distance</t>
-  </si>
-  <si>
-    <t>yes</t>
   </si>
   <si>
     <t>cal</t>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>6p</t>
+  </si>
+  <si>
+    <t>floor in</t>
   </si>
 </sst>
 </file>
@@ -630,14 +630,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C9505C6-8C48-4F60-8F09-94A266D14E03}">
-  <dimension ref="A1:E1048576"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="11.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -651,10 +651,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -667,11 +670,14 @@
       <c r="D2">
         <v>1270</v>
       </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -684,11 +690,14 @@
       <c r="D3">
         <v>1270</v>
       </c>
-      <c r="E3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -701,11 +710,14 @@
       <c r="D4">
         <v>1270</v>
       </c>
-      <c r="E4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -718,11 +730,14 @@
       <c r="D5">
         <v>1270</v>
       </c>
-      <c r="E5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
@@ -735,11 +750,14 @@
       <c r="D6">
         <v>1270</v>
       </c>
-      <c r="E6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
@@ -752,11 +770,14 @@
       <c r="D7">
         <v>1270</v>
       </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
@@ -769,8 +790,11 @@
       <c r="D8">
         <v>1270</v>
       </c>
-      <c r="E8" t="s">
-        <v>4</v>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="1048576" spans="5:5" x14ac:dyDescent="0.45">
@@ -790,95 +814,95 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="N2" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="C3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="E3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="G3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="I3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="K3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="8" t="s">
-        <v>14</v>
-      </c>
       <c r="M3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N3" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16.899999999999999" thickBot="1" x14ac:dyDescent="0.5">

</xml_diff>